<commit_message>
Tracker + handoff: first real Windows numbers (CI run 2)
Measured on the GitHub Windows runner's NTFS C: (15-10-2026): raw MFT read of 1,201,506 files
and 208,449 folders (131 GB) in 10.3 s; MFT vs Windows' own listing on Program Files 304,060
entries with 0 differences (listing 100 s vs MFT 3.8 s); System32 13 of 23,053 differ, all
live log files whose folder-listing entry is stale while Windows writes them; Quick scan of C:
40.5 s total; Excel + CSV 1.41M rows in 21.9 s; 60 engine tests pass on Windows; exe 15.5 MB.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JJft2CDRr1K9DPQpRfofKc
</commit_message>
<xml_diff>
--- a/drive-scanner/TRACKER.xlsx
+++ b/drive-scanner/TRACKER.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -528,9 +528,9 @@
           <t>2. Fast metadata scan: NTFS MFT reader (needs admin)</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -538,14 +538,10 @@
           <t>15-10-2026</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>CI run</t>
-        </is>
-      </c>
+      <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>3 GB NTFS image, 67,103 entries: 0 differences vs folder walk; 0.11 s vs 2.69 s. Hard cases proven: 221 hard links via $ATTRIBUTE_LIST, DOS names hidden, Hindi/Marathi names, sparse, fragmented. Raw \\.\C: path on Windows: CI pending.</t>
+          <t>3 GB NTFS image, 67,103 entries: 0 differences vs folder walk; 0.11 s vs 2.69 s. Hard cases proven: 221 hard links via $ATTRIBUTE_LIST, DOS names hidden, Hindi/Marathi names, sparse, fragmented. REAL WINDOWS (GitHub runner C:, run 2): 1,201,506 files + 208,449 folders, 131 GB, MFT read in 10.3 s.</t>
         </is>
       </c>
     </row>
@@ -555,9 +551,9 @@
           <t>3. Fallback scan: parallel folder walk (exFAT/FAT32, no admin, network)</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -565,14 +561,10 @@
           <t>15-10-2026</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>CI run</t>
-        </is>
-      </c>
+      <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Proven on Linux. Windows FindFirstFileExW path compiles; CI compare on C:\Program Files pending.</t>
+          <t>REAL WINDOWS: Program Files 304,060 entries, walk 100 s vs MFT 3.8 s (whole volume), 0 differences. System32 23,053 entries: 13 live log files differ (folder listing stale while Windows writes them; MFT is the true value).</t>
         </is>
       </c>
     </row>
@@ -982,12 +974,12 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>CI run</t>
+          <t>Ravi's PC</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Proven on Linux build with real engine. Windows exe: CI pending.</t>
+          <t>Proven on Linux build with real engine (mouse click-through). Windows exe BUILT (15.5 MB); not yet opened on Ravi's PC.</t>
         </is>
       </c>
     </row>
@@ -997,20 +989,20 @@
           <t>21. Windows build (GitHub Actions, portable exe, no shortcuts)</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>CI run</t>
-        </is>
-      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>15-10-2026</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Workflow written; first run starts on push.</t>
+          <t>Run 2 green: artifact AVNI-Drive-Scanner-windows-x64, 15.5 MB, sha256 53BCF921F67C9CB0815DB9103E96356B716B75C169E6FA2A1775AE252E930EE9. All 60 engine tests pass on Windows.</t>
         </is>
       </c>
     </row>
@@ -1020,20 +1012,20 @@
           <t>22. Real-runtime check on Windows NTFS (CI runner C:)</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr"/>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>CI run</t>
-        </is>
-      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>15-10-2026</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>MFT vs Windows listing on Program Files + System32, timed Quick scan.</t>
+          <t>Quick scan of C: (1.2M files, 131 GB, SSD): metadata 4.5 s, total 40.5 s, 467 duplicate sets confirmed, 800 copies kept by the tree law. Excel + CSV 1.41M rows in 21.9 s.</t>
         </is>
       </c>
     </row>
@@ -1182,25 +1174,52 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
+          <t>30. Finished files, in-app preview, in-app report/log viewer (Ravi: show everything inside the app)</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>15-10-2026</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>today</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Engine + commands done and tested (3 tests). Screens in progress.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
           <t>29. MOVED ledger (D:\AVNI DATA\_MOVED LEDGER\moved-ledger.csv)</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>15-10-2026</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>15-10-2026</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Ravi's PC</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>Written when that folder exists. NOT RUN on Ravi's PC.</t>
         </is>

</xml_diff>